<commit_message>
Update historic location descriptions to tidy up site
</commit_message>
<xml_diff>
--- a/data/locations.xlsx
+++ b/data/locations.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10830"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10909"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/james/pCloud Drive/Backups/Dropbox - James Richardson - 2026-01-30/Documents/Ferns/Flora of Todmorden/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/james/Projects/todmorden-ferns/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A56FE164-8F9A-1046-893B-2CE4CD0FC97A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB64294E-C618-8C43-8160-4F87A64E3010}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12500" yWindow="1180" windowWidth="28040" windowHeight="17440" xr2:uid="{0C0E0C07-E18F-6946-8B13-627C76AFCE0E}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="44800" windowHeight="22840" xr2:uid="{0C0E0C07-E18F-6946-8B13-627C76AFCE0E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="455" uniqueCount="185">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="455" uniqueCount="182">
   <si>
     <t>Equisetum telmateia</t>
   </si>
@@ -50,9 +50,6 @@
     <t>Above Hey Rake Farm</t>
   </si>
   <si>
-    <t>High Greenwood Wood</t>
-  </si>
-  <si>
     <t>Staups Clough</t>
   </si>
   <si>
@@ -110,9 +107,6 @@
     <t>Cryptogramma crispa</t>
   </si>
   <si>
-    <t>Scarth-rake, Cliviger.</t>
-  </si>
-  <si>
     <t>Ratton Clough, Cliviger</t>
   </si>
   <si>
@@ -164,9 +158,6 @@
     <t>Gymnocarpium dryopteris</t>
   </si>
   <si>
-    <t>Dodbottom;</t>
-  </si>
-  <si>
     <t>Nearly all shady woods of district</t>
   </si>
   <si>
@@ -182,9 +173,6 @@
     <t>Oreopteris limbosperma</t>
   </si>
   <si>
-    <t>On most of the mountainous heaths in the district. Seldom seen below 800 feet of altitude.</t>
-  </si>
-  <si>
     <t>Lastrea filix-mas</t>
   </si>
   <si>
@@ -245,18 +233,9 @@
     <t>Asplenium adiantum-nigrum</t>
   </si>
   <si>
-    <t>near Mount Skip</t>
-  </si>
-  <si>
-    <t>near Hebden Bridge</t>
-  </si>
-  <si>
     <t>Scout, Harley-wood</t>
   </si>
   <si>
-    <t>now rare</t>
-  </si>
-  <si>
     <t>Asplenium trichomanes</t>
   </si>
   <si>
@@ -275,9 +254,6 @@
     <t>rare</t>
   </si>
   <si>
-    <t>rare in locations</t>
-  </si>
-  <si>
     <t>Asplenium viride</t>
   </si>
   <si>
@@ -353,9 +329,6 @@
     <t>above Allescholes, on the moor</t>
   </si>
   <si>
-    <t>now very rare</t>
-  </si>
-  <si>
     <t>Fields near Speed clough, Harley-wood</t>
   </si>
   <si>
@@ -389,14 +362,6 @@
     <t>Chara vulgaris</t>
   </si>
   <si>
-    <t>in the pond near Holmes Chapel, Cliviger</t>
-  </si>
-  <si>
-    <t>About a quarter of a mile below Shedding House on
-the opposite side of the brook, and among the heaps of rubble
-stones.</t>
-  </si>
-  <si>
     <t>Type</t>
   </si>
   <si>
@@ -415,18 +380,12 @@
     <t>Pteridium aquilinum</t>
   </si>
   <si>
-    <t>Woods and heaths; common throughout district</t>
-  </si>
-  <si>
     <t>destroyed by moor fire</t>
   </si>
   <si>
     <t>Dryopteris affinis</t>
   </si>
   <si>
-    <t>many rocky ravines of the district</t>
-  </si>
-  <si>
     <t>Dryopteris oreades</t>
   </si>
   <si>
@@ -499,9 +458,6 @@
     <t>shedding_lime_kilns</t>
   </si>
   <si>
-    <t>below the Ridge public-house</t>
-  </si>
-  <si>
     <t>below_the_ridge_ph</t>
   </si>
   <si>
@@ -596,6 +552,39 @@
   </si>
   <si>
     <t>ponds_near_holmes_chapel</t>
+  </si>
+  <si>
+    <t>High Greenwood</t>
+  </si>
+  <si>
+    <t>Scarth-rake, Cliviger</t>
+  </si>
+  <si>
+    <t>Dodbottom</t>
+  </si>
+  <si>
+    <t>About a quarter of a mile below Shedding House on the opposite side of the brook, and among the heaps of rubble stones</t>
+  </si>
+  <si>
+    <t>On most of the mountainous heaths in the district. Seldom seen below 800 feet of altitude</t>
+  </si>
+  <si>
+    <t>In the pond near Holmes Chapel, Cliviger</t>
+  </si>
+  <si>
+    <t>Woods and heaths - common throughout district</t>
+  </si>
+  <si>
+    <t>Many rocky ravines of the district</t>
+  </si>
+  <si>
+    <t>Below the Ridge public-house</t>
+  </si>
+  <si>
+    <t>Near Mount Skip</t>
+  </si>
+  <si>
+    <t>Near Hebden Bridge</t>
   </si>
 </sst>
 </file>
@@ -992,7 +981,7 @@
   <cols>
     <col min="1" max="1" width="24" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
-    <col min="5" max="5" width="27.1640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="33.33203125" customWidth="1"/>
     <col min="6" max="6" width="17" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="19" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="12.83203125" bestFit="1" customWidth="1"/>
@@ -1001,34 +990,34 @@
   <sheetData>
     <row r="1" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="F1" s="1" t="s">
-        <v>12</v>
-      </c>
       <c r="G1" s="1" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>118</v>
+        <v>107</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>177</v>
+        <v>163</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>178</v>
+        <v>164</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="17" x14ac:dyDescent="0.2">
@@ -1047,10 +1036,10 @@
       </c>
       <c r="F2" s="1"/>
       <c r="H2" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="I2" t="s">
-        <v>129</v>
+        <v>116</v>
       </c>
       <c r="J2">
         <v>31</v>
@@ -1068,14 +1057,14 @@
         <v>-2.042748</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>3</v>
+        <v>171</v>
       </c>
       <c r="F3" s="1"/>
       <c r="H3" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="I3" t="s">
-        <v>131</v>
+        <v>118</v>
       </c>
       <c r="J3">
         <v>31</v>
@@ -1093,14 +1082,14 @@
         <v>-2.0704132</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F4" s="1"/>
       <c r="H4" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="I4" t="s">
-        <v>130</v>
+        <v>117</v>
       </c>
       <c r="J4">
         <v>31</v>
@@ -1108,7 +1097,7 @@
     </row>
     <row r="5" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B5" s="1"/>
       <c r="C5" s="1">
@@ -1118,14 +1107,14 @@
         <v>-2.1654163999999998</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F5" s="1"/>
       <c r="H5" t="s">
+        <v>108</v>
+      </c>
+      <c r="I5" t="s">
         <v>119</v>
-      </c>
-      <c r="I5" t="s">
-        <v>132</v>
       </c>
       <c r="J5">
         <v>31</v>
@@ -1133,19 +1122,19 @@
     </row>
     <row r="6" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C6" s="1"/>
       <c r="D6" s="1"/>
       <c r="E6" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F6" s="1"/>
       <c r="H6" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="J6">
         <v>31</v>
@@ -1153,19 +1142,19 @@
     </row>
     <row r="7" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C7" s="1"/>
       <c r="D7" s="1"/>
       <c r="E7" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F7" s="1"/>
       <c r="H7" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="J7">
         <v>31</v>
@@ -1173,21 +1162,21 @@
     </row>
     <row r="8" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C8" s="1"/>
       <c r="D8" s="1"/>
       <c r="E8" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H8" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="J8">
         <v>31</v>
@@ -1195,7 +1184,7 @@
     </row>
     <row r="9" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B9" s="1"/>
       <c r="C9" s="1">
@@ -1205,16 +1194,16 @@
         <v>-2.1718850000000001</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>23</v>
+        <v>172</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H9" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="I9" t="s">
-        <v>133</v>
+        <v>120</v>
       </c>
       <c r="J9">
         <v>31</v>
@@ -1222,7 +1211,7 @@
     </row>
     <row r="10" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B10" s="1"/>
       <c r="C10" s="1">
@@ -1232,16 +1221,16 @@
         <v>-2.18194</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H10" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="I10" t="s">
-        <v>134</v>
+        <v>121</v>
       </c>
       <c r="J10">
         <v>31</v>
@@ -1249,7 +1238,7 @@
     </row>
     <row r="11" spans="1:10" ht="34" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B11" s="1"/>
       <c r="C11" s="1">
@@ -1259,16 +1248,16 @@
         <v>-2.174137</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H11" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="I11" t="s">
-        <v>135</v>
+        <v>122</v>
       </c>
       <c r="J11">
         <v>31</v>
@@ -1276,7 +1265,7 @@
     </row>
     <row r="12" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B12" s="1"/>
       <c r="C12" s="1">
@@ -1286,16 +1275,16 @@
         <v>-2.1684223</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H12" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="I12" t="s">
-        <v>136</v>
+        <v>123</v>
       </c>
       <c r="J12">
         <v>31</v>
@@ -1303,19 +1292,19 @@
     </row>
     <row r="13" spans="1:10" ht="34" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C13" s="1"/>
       <c r="D13" s="1"/>
       <c r="E13" s="1" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="F13" s="1"/>
       <c r="H13" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="J13">
         <v>31</v>
@@ -1323,7 +1312,7 @@
     </row>
     <row r="14" spans="1:10" ht="34" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B14" s="1"/>
       <c r="C14" s="1">
@@ -1333,16 +1322,16 @@
         <v>-2.0919219</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="H14" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="I14" t="s">
-        <v>137</v>
+        <v>124</v>
       </c>
       <c r="J14">
         <v>31</v>
@@ -1350,7 +1339,7 @@
     </row>
     <row r="15" spans="1:10" ht="34" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B15" s="1"/>
       <c r="C15" s="1">
@@ -1360,16 +1349,16 @@
         <v>-2.0436529999999999</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="H15" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="I15" t="s">
-        <v>138</v>
+        <v>125</v>
       </c>
       <c r="J15">
         <v>31</v>
@@ -1377,7 +1366,7 @@
     </row>
     <row r="16" spans="1:10" ht="34" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B16" s="1"/>
       <c r="C16" s="1">
@@ -1387,16 +1376,16 @@
         <v>-2.1937121999999998</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="H16" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="I16" t="s">
-        <v>139</v>
+        <v>126</v>
       </c>
       <c r="J16">
         <v>31</v>
@@ -1404,7 +1393,7 @@
     </row>
     <row r="17" spans="1:10" ht="34" x14ac:dyDescent="0.2">
       <c r="A17" s="1" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B17" s="1"/>
       <c r="C17" s="1">
@@ -1414,16 +1403,16 @@
         <v>-2.1185657999999998</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="H17" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="I17" t="s">
-        <v>140</v>
+        <v>127</v>
       </c>
       <c r="J17">
         <v>31</v>
@@ -1431,7 +1420,7 @@
     </row>
     <row r="18" spans="1:10" ht="34" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B18" s="1"/>
       <c r="C18" s="1">
@@ -1441,16 +1430,16 @@
         <v>-2.1871551</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="H18" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="I18" t="s">
-        <v>141</v>
+        <v>128</v>
       </c>
       <c r="J18">
         <v>31</v>
@@ -1458,7 +1447,7 @@
     </row>
     <row r="19" spans="1:10" ht="34" x14ac:dyDescent="0.2">
       <c r="A19" s="1" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B19" s="1"/>
       <c r="C19" s="1">
@@ -1468,16 +1457,16 @@
         <v>-2.1235843000000001</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="H19" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="I19" t="s">
-        <v>142</v>
+        <v>129</v>
       </c>
       <c r="J19">
         <v>31</v>
@@ -1485,7 +1474,7 @@
     </row>
     <row r="20" spans="1:10" ht="34" x14ac:dyDescent="0.2">
       <c r="A20" s="1" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B20" s="1"/>
       <c r="C20" s="1">
@@ -1495,16 +1484,16 @@
         <v>-2.1466509999999999</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="H20" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="I20" t="s">
-        <v>143</v>
+        <v>130</v>
       </c>
       <c r="J20">
         <v>31</v>
@@ -1512,21 +1501,21 @@
     </row>
     <row r="21" spans="1:10" ht="34" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C21" s="1"/>
       <c r="D21" s="1"/>
       <c r="E21" s="1" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="H21" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="J21">
         <v>31</v>
@@ -1534,7 +1523,7 @@
     </row>
     <row r="22" spans="1:10" ht="34" x14ac:dyDescent="0.2">
       <c r="A22" s="1" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B22" s="1"/>
       <c r="C22" s="1">
@@ -1544,16 +1533,16 @@
         <v>-2.0436529999999999</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="H22" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="I22" t="s">
-        <v>138</v>
+        <v>125</v>
       </c>
       <c r="J22">
         <v>31</v>
@@ -1561,7 +1550,7 @@
     </row>
     <row r="23" spans="1:10" ht="34" x14ac:dyDescent="0.2">
       <c r="A23" s="1" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B23" s="1"/>
       <c r="C23" s="1">
@@ -1571,16 +1560,16 @@
         <v>-2.1960535999999999</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>41</v>
+        <v>173</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="H23" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="I23" t="s">
-        <v>144</v>
+        <v>131</v>
       </c>
       <c r="J23">
         <v>31</v>
@@ -1588,7 +1577,7 @@
     </row>
     <row r="24" spans="1:10" ht="34" x14ac:dyDescent="0.2">
       <c r="A24" s="1" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B24" s="1"/>
       <c r="C24" s="1">
@@ -1598,16 +1587,16 @@
         <v>-2.0704132</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="H24" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="I24" t="s">
-        <v>130</v>
+        <v>117</v>
       </c>
       <c r="J24">
         <v>31</v>
@@ -1615,7 +1604,7 @@
     </row>
     <row r="25" spans="1:10" ht="34" x14ac:dyDescent="0.2">
       <c r="A25" s="1" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B25" s="1"/>
       <c r="C25" s="1">
@@ -1625,16 +1614,16 @@
         <v>-2.1937121999999998</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="H25" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="I25" t="s">
-        <v>139</v>
+        <v>126</v>
       </c>
       <c r="J25">
         <v>31</v>
@@ -1642,29 +1631,29 @@
     </row>
     <row r="26" spans="1:10" ht="34" x14ac:dyDescent="0.2">
       <c r="A26" s="1" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C26" s="1"/>
       <c r="D26" s="1"/>
       <c r="E26" s="1" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="H26" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="J26">
         <v>31</v>
       </c>
     </row>
-    <row r="27" spans="1:10" ht="85" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:10" ht="68" x14ac:dyDescent="0.2">
       <c r="A27" s="1" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="B27" s="1"/>
       <c r="C27" s="1">
@@ -1674,16 +1663,16 @@
         <v>-2.1662952999999998</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>117</v>
+        <v>174</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="H27" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="I27" t="s">
-        <v>145</v>
+        <v>132</v>
       </c>
       <c r="J27">
         <v>32</v>
@@ -1691,21 +1680,21 @@
     </row>
     <row r="28" spans="1:10" ht="51" x14ac:dyDescent="0.2">
       <c r="A28" s="1" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C28" s="1"/>
       <c r="D28" s="1"/>
       <c r="E28" s="1" t="s">
-        <v>47</v>
+        <v>175</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="H28" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="J28">
         <v>32</v>
@@ -1713,21 +1702,21 @@
     </row>
     <row r="29" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="A29" s="1" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C29" s="2"/>
       <c r="D29" s="2"/>
       <c r="E29" s="2" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="F29" s="1" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="H29" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="J29">
         <v>32</v>
@@ -1735,21 +1724,21 @@
     </row>
     <row r="30" spans="1:10" ht="34" x14ac:dyDescent="0.2">
       <c r="A30" s="1" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C30" s="2"/>
       <c r="D30" s="2"/>
       <c r="E30" s="2" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="F30" s="1" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="H30" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="J30">
         <v>32</v>
@@ -1757,7 +1746,7 @@
     </row>
     <row r="31" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="A31" s="1" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="C31">
         <v>53.728571000000002</v>
@@ -1766,13 +1755,13 @@
         <v>-2.1089715</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="H31" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="I31" t="s">
-        <v>146</v>
+        <v>133</v>
       </c>
       <c r="J31">
         <v>33</v>
@@ -1780,7 +1769,7 @@
     </row>
     <row r="32" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="A32" s="1" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="C32">
         <v>53.724857999999998</v>
@@ -1789,13 +1778,13 @@
         <v>-2.0951558000000001</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="H32" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="I32" t="s">
-        <v>147</v>
+        <v>134</v>
       </c>
       <c r="J32">
         <v>33</v>
@@ -1803,7 +1792,7 @@
     </row>
     <row r="33" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="A33" s="1" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="C33" s="1">
         <v>53.770833000000003</v>
@@ -1812,13 +1801,13 @@
         <v>-2.0436529999999999</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="H33" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="I33" t="s">
-        <v>138</v>
+        <v>125</v>
       </c>
       <c r="J33">
         <v>33</v>
@@ -1826,13 +1815,13 @@
     </row>
     <row r="34" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="A34" s="1" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="H34" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="J34">
         <v>33</v>
@@ -1840,7 +1829,7 @@
     </row>
     <row r="35" spans="1:10" ht="34" x14ac:dyDescent="0.2">
       <c r="A35" s="1" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="C35">
         <v>53.764629999999997</v>
@@ -1849,13 +1838,13 @@
         <v>-2.1619999999999999</v>
       </c>
       <c r="E35" s="1" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="H35" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="I35" t="s">
-        <v>148</v>
+        <v>135</v>
       </c>
       <c r="J35">
         <v>33</v>
@@ -1863,7 +1852,7 @@
     </row>
     <row r="36" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="A36" s="1" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="C36" s="1">
         <v>53.754627999999997</v>
@@ -1872,13 +1861,13 @@
         <v>-2.1937121999999998</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="H36" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="I36" t="s">
-        <v>139</v>
+        <v>126</v>
       </c>
       <c r="J36">
         <v>33</v>
@@ -1886,7 +1875,7 @@
     </row>
     <row r="37" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="A37" s="1" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="C37">
         <v>53.690149699999999</v>
@@ -1895,13 +1884,13 @@
         <v>-2.1151597</v>
       </c>
       <c r="E37" s="1" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="H37" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="I37" t="s">
-        <v>149</v>
+        <v>136</v>
       </c>
       <c r="J37">
         <v>33</v>
@@ -1909,7 +1898,7 @@
     </row>
     <row r="38" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="A38" s="1" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="C38">
         <v>53.721606000000001</v>
@@ -1918,13 +1907,13 @@
         <v>-2.1190077999999999</v>
       </c>
       <c r="E38" s="1" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="H38" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="I38" t="s">
-        <v>150</v>
+        <v>137</v>
       </c>
       <c r="J38">
         <v>33</v>
@@ -1932,7 +1921,7 @@
     </row>
     <row r="39" spans="1:10" ht="34" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="C39">
         <v>53.762680000000003</v>
@@ -1941,13 +1930,13 @@
         <v>-2.1602999999999999</v>
       </c>
       <c r="E39" s="1" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="H39" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="I39" t="s">
-        <v>151</v>
+        <v>138</v>
       </c>
       <c r="J39">
         <v>33</v>
@@ -1955,7 +1944,7 @@
     </row>
     <row r="40" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="C40">
         <v>53.778702000000003</v>
@@ -1964,13 +1953,13 @@
         <v>-2.0793341000000001</v>
       </c>
       <c r="E40" s="1" t="s">
-        <v>152</v>
+        <v>179</v>
       </c>
       <c r="H40" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="I40" t="s">
-        <v>153</v>
+        <v>139</v>
       </c>
       <c r="J40">
         <v>33</v>
@@ -1978,7 +1967,7 @@
     </row>
     <row r="41" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="C41">
         <v>53.751420000000003</v>
@@ -1987,13 +1976,13 @@
         <v>-2.2123900000000001</v>
       </c>
       <c r="E41" s="1" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="H41" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="I41" t="s">
-        <v>154</v>
+        <v>140</v>
       </c>
       <c r="J41">
         <v>33</v>
@@ -2001,7 +1990,7 @@
     </row>
     <row r="42" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="C42" s="1">
         <v>53.754627999999997</v>
@@ -2010,13 +1999,13 @@
         <v>-2.1937121999999998</v>
       </c>
       <c r="E42" s="1" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="H42" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="I42" t="s">
-        <v>139</v>
+        <v>126</v>
       </c>
       <c r="J42">
         <v>33</v>
@@ -2024,7 +2013,7 @@
     </row>
     <row r="43" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="C43" s="1">
         <v>53.741953600000002</v>
@@ -2033,13 +2022,13 @@
         <v>-2.1871551</v>
       </c>
       <c r="E43" s="1" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="H43" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="I43" t="s">
-        <v>141</v>
+        <v>128</v>
       </c>
       <c r="J43">
         <v>33</v>
@@ -2047,16 +2036,16 @@
     </row>
     <row r="44" spans="1:10" ht="34" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="B44" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E44" s="1" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="H44" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="J44">
         <v>33</v>
@@ -2064,7 +2053,7 @@
     </row>
     <row r="45" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="C45">
         <v>53.743994000000001</v>
@@ -2073,16 +2062,16 @@
         <v>-1.9882738</v>
       </c>
       <c r="E45" s="1" t="s">
-        <v>68</v>
+        <v>180</v>
       </c>
       <c r="G45" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="H45" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="I45" t="s">
-        <v>155</v>
+        <v>141</v>
       </c>
       <c r="J45">
         <v>34</v>
@@ -2090,16 +2079,16 @@
     </row>
     <row r="46" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="E46" s="1" t="s">
-        <v>69</v>
+        <v>181</v>
       </c>
       <c r="G46" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="H46" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="J46">
         <v>34</v>
@@ -2107,7 +2096,7 @@
     </row>
     <row r="47" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="C47">
         <v>53.729149499999998</v>
@@ -2116,16 +2105,16 @@
         <v>-2.1060009000000002</v>
       </c>
       <c r="E47" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="G47" t="s">
         <v>70</v>
       </c>
-      <c r="G47" t="s">
-        <v>71</v>
-      </c>
       <c r="H47" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="I47" t="s">
-        <v>156</v>
+        <v>142</v>
       </c>
       <c r="J47">
         <v>34</v>
@@ -2133,7 +2122,7 @@
     </row>
     <row r="48" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="C48" s="1">
         <v>53.769137999999998</v>
@@ -2142,16 +2131,16 @@
         <v>-2.1654163999999998</v>
       </c>
       <c r="E48" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G48" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="H48" t="s">
+        <v>108</v>
+      </c>
+      <c r="I48" t="s">
         <v>119</v>
-      </c>
-      <c r="I48" t="s">
-        <v>132</v>
       </c>
       <c r="J48">
         <v>34</v>
@@ -2159,7 +2148,7 @@
     </row>
     <row r="49" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="C49" s="1">
         <v>53.741953600000002</v>
@@ -2168,33 +2157,33 @@
         <v>-2.1871551</v>
       </c>
       <c r="E49" s="1" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="G49" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="H49" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="I49" t="s">
-        <v>141</v>
+        <v>128</v>
       </c>
       <c r="J49">
         <v>34</v>
       </c>
     </row>
-    <row r="50" spans="1:10" ht="34" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="E50" s="1" t="s">
-        <v>83</v>
+        <v>75</v>
       </c>
       <c r="G50" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="H50" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="J50">
         <v>34</v>
@@ -2202,7 +2191,7 @@
     </row>
     <row r="51" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="C51" s="1">
         <v>53.769137999999998</v>
@@ -2211,16 +2200,16 @@
         <v>-2.1654163999999998</v>
       </c>
       <c r="E51" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G51" t="s">
-        <v>78</v>
+        <v>70</v>
       </c>
       <c r="H51" t="s">
+        <v>108</v>
+      </c>
+      <c r="I51" t="s">
         <v>119</v>
-      </c>
-      <c r="I51" t="s">
-        <v>132</v>
       </c>
       <c r="J51">
         <v>34</v>
@@ -2228,7 +2217,7 @@
     </row>
     <row r="52" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="C52">
         <v>53.775243000000003</v>
@@ -2237,24 +2226,24 @@
         <v>-2.1550193000000002</v>
       </c>
       <c r="E52" s="1" t="s">
-        <v>73</v>
+        <v>66</v>
       </c>
       <c r="G52" t="s">
-        <v>78</v>
+        <v>70</v>
       </c>
       <c r="H52" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="I52" t="s">
-        <v>157</v>
+        <v>143</v>
       </c>
       <c r="J52">
         <v>34</v>
       </c>
     </row>
-    <row r="53" spans="1:10" ht="34" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="C53">
         <v>53.748814000000003</v>
@@ -2263,16 +2252,16 @@
         <v>-2.1984729999999999</v>
       </c>
       <c r="E53" s="1" t="s">
-        <v>74</v>
+        <v>67</v>
       </c>
       <c r="G53" t="s">
-        <v>78</v>
+        <v>70</v>
       </c>
       <c r="H53" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="I53" t="s">
-        <v>144</v>
+        <v>131</v>
       </c>
       <c r="J53">
         <v>34</v>
@@ -2280,7 +2269,7 @@
     </row>
     <row r="54" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="C54" s="1">
         <v>53.741953600000002</v>
@@ -2289,16 +2278,16 @@
         <v>-2.1871551</v>
       </c>
       <c r="E54" s="1" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="G54" t="s">
-        <v>78</v>
+        <v>70</v>
       </c>
       <c r="H54" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="I54" t="s">
-        <v>141</v>
+        <v>128</v>
       </c>
       <c r="J54">
         <v>34</v>
@@ -2306,7 +2295,7 @@
     </row>
     <row r="55" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="C55" s="1">
         <v>53.774380399999998</v>
@@ -2315,16 +2304,16 @@
         <v>-2.042748</v>
       </c>
       <c r="E55" s="1" t="s">
-        <v>3</v>
+        <v>171</v>
       </c>
       <c r="G55" t="s">
-        <v>78</v>
+        <v>70</v>
       </c>
       <c r="H55" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="I55" t="s">
-        <v>131</v>
+        <v>118</v>
       </c>
       <c r="J55">
         <v>34</v>
@@ -2332,7 +2321,7 @@
     </row>
     <row r="56" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="C56" s="1">
         <v>53.770833000000003</v>
@@ -2341,16 +2330,16 @@
         <v>-2.0436529999999999</v>
       </c>
       <c r="E56" s="1" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="G56" t="s">
-        <v>78</v>
+        <v>70</v>
       </c>
       <c r="H56" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="I56" t="s">
-        <v>138</v>
+        <v>125</v>
       </c>
       <c r="J56">
         <v>34</v>
@@ -2358,7 +2347,7 @@
     </row>
     <row r="57" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="C57" s="3">
         <v>53.729149499999998</v>
@@ -2367,16 +2356,16 @@
         <v>-2.1060009000000002</v>
       </c>
       <c r="E57" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="G57" t="s">
         <v>70</v>
       </c>
-      <c r="G57" t="s">
-        <v>78</v>
-      </c>
       <c r="H57" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="I57" t="s">
-        <v>156</v>
+        <v>142</v>
       </c>
       <c r="J57">
         <v>34</v>
@@ -2384,7 +2373,7 @@
     </row>
     <row r="58" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="C58" s="1">
         <v>53.746470000000002</v>
@@ -2393,16 +2382,16 @@
         <v>-2.0294002999999998</v>
       </c>
       <c r="E58" s="1" t="s">
-        <v>75</v>
+        <v>68</v>
       </c>
       <c r="G58" t="s">
-        <v>78</v>
+        <v>70</v>
       </c>
       <c r="H58" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="I58" t="s">
-        <v>158</v>
+        <v>144</v>
       </c>
       <c r="J58">
         <v>34</v>
@@ -2410,16 +2399,16 @@
     </row>
     <row r="59" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="E59" s="1" t="s">
-        <v>76</v>
+        <v>69</v>
       </c>
       <c r="G59" t="s">
-        <v>78</v>
+        <v>70</v>
       </c>
       <c r="H59" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="J59">
         <v>34</v>
@@ -2427,7 +2416,7 @@
     </row>
     <row r="60" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
-        <v>79</v>
+        <v>71</v>
       </c>
       <c r="C60">
         <v>53.70664</v>
@@ -2436,16 +2425,16 @@
         <v>-2.1226742999999999</v>
       </c>
       <c r="E60" s="1" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="G60" t="s">
-        <v>82</v>
+        <v>74</v>
       </c>
       <c r="H60" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="I60" t="s">
-        <v>159</v>
+        <v>145</v>
       </c>
       <c r="J60">
         <v>34</v>
@@ -2453,7 +2442,7 @@
     </row>
     <row r="61" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
-        <v>79</v>
+        <v>71</v>
       </c>
       <c r="C61" s="1">
         <v>53.706695000000003</v>
@@ -2462,16 +2451,16 @@
         <v>-2.1235843000000001</v>
       </c>
       <c r="E61" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="G61" t="s">
-        <v>82</v>
+        <v>74</v>
       </c>
       <c r="H61" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="I61" t="s">
-        <v>142</v>
+        <v>129</v>
       </c>
       <c r="J61">
         <v>34</v>
@@ -2479,7 +2468,7 @@
     </row>
     <row r="62" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
-        <v>79</v>
+        <v>71</v>
       </c>
       <c r="C62">
         <v>53.690149699999999</v>
@@ -2488,16 +2477,16 @@
         <v>-2.1151597</v>
       </c>
       <c r="E62" s="1" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="G62" t="s">
-        <v>82</v>
+        <v>74</v>
       </c>
       <c r="H62" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="I62" t="s">
-        <v>149</v>
+        <v>136</v>
       </c>
       <c r="J62">
         <v>34</v>
@@ -2505,7 +2494,7 @@
     </row>
     <row r="63" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
-        <v>79</v>
+        <v>71</v>
       </c>
       <c r="C63">
         <v>53.725749</v>
@@ -2514,16 +2503,16 @@
         <v>-2.1495522</v>
       </c>
       <c r="E63" s="1" t="s">
-        <v>81</v>
+        <v>73</v>
       </c>
       <c r="G63" t="s">
-        <v>82</v>
+        <v>74</v>
       </c>
       <c r="H63" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="I63" t="s">
-        <v>160</v>
+        <v>146</v>
       </c>
       <c r="J63">
         <v>34</v>
@@ -2531,7 +2520,7 @@
     </row>
     <row r="64" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
-        <v>84</v>
+        <v>76</v>
       </c>
       <c r="C64" s="1">
         <v>53.746470000000002</v>
@@ -2540,16 +2529,16 @@
         <v>-2.0294002999999998</v>
       </c>
       <c r="E64" s="1" t="s">
-        <v>85</v>
+        <v>77</v>
       </c>
       <c r="G64" t="s">
-        <v>87</v>
+        <v>79</v>
       </c>
       <c r="H64" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="I64" t="s">
-        <v>161</v>
+        <v>147</v>
       </c>
       <c r="J64">
         <v>34</v>
@@ -2557,7 +2546,7 @@
     </row>
     <row r="65" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
-        <v>84</v>
+        <v>76</v>
       </c>
       <c r="C65">
         <v>53.770164000000001</v>
@@ -2566,16 +2555,16 @@
         <v>-2.2068927</v>
       </c>
       <c r="E65" s="1" t="s">
-        <v>86</v>
+        <v>78</v>
       </c>
       <c r="G65" t="s">
-        <v>77</v>
+        <v>70</v>
       </c>
       <c r="H65" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="I65" t="s">
-        <v>162</v>
+        <v>148</v>
       </c>
       <c r="J65">
         <v>34</v>
@@ -2583,7 +2572,7 @@
     </row>
     <row r="66" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="C66" s="1">
         <v>53.770833000000003</v>
@@ -2592,19 +2581,19 @@
         <v>-2.0436529999999999</v>
       </c>
       <c r="E66" s="1" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="F66" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="G66" t="s">
-        <v>77</v>
+        <v>70</v>
       </c>
       <c r="H66" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="I66" t="s">
-        <v>138</v>
+        <v>125</v>
       </c>
       <c r="J66">
         <v>34</v>
@@ -2612,7 +2601,7 @@
     </row>
     <row r="67" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="C67">
         <v>53.775243000000003</v>
@@ -2621,19 +2610,19 @@
         <v>-2.1550193000000002</v>
       </c>
       <c r="E67" s="1" t="s">
-        <v>73</v>
+        <v>66</v>
       </c>
       <c r="F67" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="G67" t="s">
-        <v>77</v>
+        <v>70</v>
       </c>
       <c r="H67" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="I67" t="s">
-        <v>157</v>
+        <v>143</v>
       </c>
       <c r="J67">
         <v>34</v>
@@ -2641,7 +2630,7 @@
     </row>
     <row r="68" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="C68">
         <v>53.724857999999998</v>
@@ -2650,19 +2639,19 @@
         <v>-2.0951558000000001</v>
       </c>
       <c r="E68" s="1" t="s">
-        <v>90</v>
+        <v>82</v>
       </c>
       <c r="F68" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="G68" t="s">
-        <v>77</v>
+        <v>70</v>
       </c>
       <c r="H68" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="I68" t="s">
-        <v>163</v>
+        <v>149</v>
       </c>
       <c r="J68">
         <v>34</v>
@@ -2670,28 +2659,28 @@
     </row>
     <row r="69" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="C69">
         <v>53.728727900000003</v>
       </c>
       <c r="D69" t="s">
-        <v>92</v>
+        <v>84</v>
       </c>
       <c r="E69" s="1" t="s">
-        <v>91</v>
+        <v>83</v>
       </c>
       <c r="F69" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="G69" t="s">
-        <v>77</v>
+        <v>70</v>
       </c>
       <c r="H69" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="I69" t="s">
-        <v>165</v>
+        <v>151</v>
       </c>
       <c r="J69">
         <v>34</v>
@@ -2699,7 +2688,7 @@
     </row>
     <row r="70" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="C70">
         <v>3.7390153000000002</v>
@@ -2708,39 +2697,39 @@
         <v>-2.0627032000000001</v>
       </c>
       <c r="E70" s="1" t="s">
-        <v>164</v>
+        <v>150</v>
       </c>
       <c r="F70" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="G70" t="s">
-        <v>77</v>
+        <v>70</v>
       </c>
       <c r="H70" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="I70" t="s">
-        <v>130</v>
+        <v>117</v>
       </c>
       <c r="J70">
         <v>34</v>
       </c>
     </row>
-    <row r="71" spans="1:10" ht="34" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
-        <v>94</v>
+        <v>86</v>
       </c>
       <c r="B71" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E71" s="1" t="s">
-        <v>95</v>
+        <v>87</v>
       </c>
       <c r="F71" t="s">
-        <v>93</v>
+        <v>85</v>
       </c>
       <c r="H71" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="J71">
         <v>34</v>
@@ -2748,7 +2737,7 @@
     </row>
     <row r="72" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="C72">
         <v>53.703311999999997</v>
@@ -2757,21 +2746,21 @@
         <v>-2.0616482999999999</v>
       </c>
       <c r="E72" s="1" t="s">
-        <v>97</v>
+        <v>89</v>
       </c>
       <c r="H72" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="I72" t="s">
-        <v>166</v>
+        <v>152</v>
       </c>
       <c r="J72">
         <v>36</v>
       </c>
     </row>
-    <row r="73" spans="1:10" ht="68" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:10" ht="51" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="C73">
         <v>53.728416000000003</v>
@@ -2780,13 +2769,13 @@
         <v>-2.1173082999999999</v>
       </c>
       <c r="E73" s="1" t="s">
-        <v>98</v>
+        <v>90</v>
       </c>
       <c r="H73" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="I73" t="s">
-        <v>167</v>
+        <v>153</v>
       </c>
       <c r="J73">
         <v>36</v>
@@ -2794,7 +2783,7 @@
     </row>
     <row r="74" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
-        <v>100</v>
+        <v>92</v>
       </c>
       <c r="C74" s="1">
         <v>53.741953600000002</v>
@@ -2803,19 +2792,19 @@
         <v>-2.1871551</v>
       </c>
       <c r="E74" s="1" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="F74" t="s">
-        <v>99</v>
+        <v>91</v>
       </c>
       <c r="G74" t="s">
-        <v>101</v>
+        <v>93</v>
       </c>
       <c r="H74" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="I74" t="s">
-        <v>141</v>
+        <v>128</v>
       </c>
       <c r="J74">
         <v>36</v>
@@ -2823,7 +2812,7 @@
     </row>
     <row r="75" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
-        <v>102</v>
+        <v>94</v>
       </c>
       <c r="C75" s="1">
         <v>53.774380399999998</v>
@@ -2832,16 +2821,16 @@
         <v>-2.042748</v>
       </c>
       <c r="E75" s="1" t="s">
-        <v>3</v>
+        <v>171</v>
       </c>
       <c r="G75" t="s">
-        <v>104</v>
+        <v>74</v>
       </c>
       <c r="H75" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="I75" t="s">
-        <v>131</v>
+        <v>118</v>
       </c>
       <c r="J75">
         <v>36</v>
@@ -2849,7 +2838,7 @@
     </row>
     <row r="76" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
-        <v>102</v>
+        <v>94</v>
       </c>
       <c r="C76">
         <v>53.678840999999998</v>
@@ -2858,16 +2847,16 @@
         <v>-2.1066463</v>
       </c>
       <c r="E76" s="1" t="s">
-        <v>103</v>
+        <v>95</v>
       </c>
       <c r="G76" t="s">
-        <v>104</v>
+        <v>74</v>
       </c>
       <c r="H76" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="I76" t="s">
-        <v>168</v>
+        <v>154</v>
       </c>
       <c r="J76">
         <v>36</v>
@@ -2875,7 +2864,7 @@
     </row>
     <row r="77" spans="1:10" ht="34" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
-        <v>108</v>
+        <v>99</v>
       </c>
       <c r="C77">
         <v>53.728416000000003</v>
@@ -2884,13 +2873,13 @@
         <v>-2.1173082999999999</v>
       </c>
       <c r="E77" s="1" t="s">
-        <v>105</v>
+        <v>96</v>
       </c>
       <c r="H77" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="I77" t="s">
-        <v>172</v>
+        <v>158</v>
       </c>
       <c r="J77">
         <v>36</v>
@@ -2898,7 +2887,7 @@
     </row>
     <row r="78" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
-        <v>108</v>
+        <v>99</v>
       </c>
       <c r="C78">
         <v>53.732166999999997</v>
@@ -2907,13 +2896,13 @@
         <v>-2.1147499000000001</v>
       </c>
       <c r="E78" s="1" t="s">
-        <v>169</v>
+        <v>155</v>
       </c>
       <c r="H78" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="I78" t="s">
-        <v>173</v>
+        <v>159</v>
       </c>
       <c r="J78">
         <v>36</v>
@@ -2921,7 +2910,7 @@
     </row>
     <row r="79" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
-        <v>108</v>
+        <v>99</v>
       </c>
       <c r="C79">
         <v>53.732166999999997</v>
@@ -2930,13 +2919,13 @@
         <v>-2.1147499000000001</v>
       </c>
       <c r="E79" s="1" t="s">
-        <v>170</v>
+        <v>156</v>
       </c>
       <c r="H79" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="I79" t="s">
-        <v>174</v>
+        <v>160</v>
       </c>
       <c r="J79">
         <v>36</v>
@@ -2944,7 +2933,7 @@
     </row>
     <row r="80" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
-        <v>108</v>
+        <v>99</v>
       </c>
       <c r="C80">
         <v>53.732166999999997</v>
@@ -2953,13 +2942,13 @@
         <v>-2.1147499000000001</v>
       </c>
       <c r="E80" s="1" t="s">
-        <v>171</v>
+        <v>157</v>
       </c>
       <c r="H80" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="I80" t="s">
-        <v>175</v>
+        <v>161</v>
       </c>
       <c r="J80">
         <v>36</v>
@@ -2967,22 +2956,22 @@
     </row>
     <row r="81" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
-        <v>108</v>
+        <v>99</v>
       </c>
       <c r="C81">
         <v>53.748199</v>
       </c>
       <c r="D81" t="s">
-        <v>107</v>
+        <v>98</v>
       </c>
       <c r="E81" s="1" t="s">
-        <v>106</v>
+        <v>97</v>
       </c>
       <c r="H81" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="I81" t="s">
-        <v>176</v>
+        <v>162</v>
       </c>
       <c r="J81">
         <v>36</v>
@@ -2990,16 +2979,16 @@
     </row>
     <row r="82" spans="1:10" ht="34" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
-        <v>109</v>
+        <v>100</v>
       </c>
       <c r="B82" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E82" s="1" t="s">
-        <v>122</v>
+        <v>111</v>
       </c>
       <c r="H82" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="J82">
         <v>36</v>
@@ -3007,7 +2996,7 @@
     </row>
     <row r="83" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
-        <v>110</v>
+        <v>101</v>
       </c>
       <c r="C83" s="1">
         <v>53.743820900000003</v>
@@ -3016,16 +3005,16 @@
         <v>-2.1466509999999999</v>
       </c>
       <c r="E83" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="G83" t="s">
-        <v>77</v>
+        <v>70</v>
       </c>
       <c r="H83" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="I83" t="s">
-        <v>143</v>
+        <v>130</v>
       </c>
       <c r="J83">
         <v>36</v>
@@ -3033,7 +3022,7 @@
     </row>
     <row r="84" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
-        <v>110</v>
+        <v>101</v>
       </c>
       <c r="C84">
         <v>53.703311999999997</v>
@@ -3042,24 +3031,24 @@
         <v>-2.0616482999999999</v>
       </c>
       <c r="E84" s="1" t="s">
-        <v>97</v>
+        <v>89</v>
       </c>
       <c r="G84" t="s">
-        <v>77</v>
+        <v>70</v>
       </c>
       <c r="H84" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="I84" t="s">
-        <v>166</v>
+        <v>152</v>
       </c>
       <c r="J84">
         <v>36</v>
       </c>
     </row>
-    <row r="85" spans="1:10" ht="34" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
-        <v>111</v>
+        <v>102</v>
       </c>
       <c r="C85">
         <v>53.737197000000002</v>
@@ -3068,16 +3057,16 @@
         <v>-2.1034240999999998</v>
       </c>
       <c r="E85" s="1" t="s">
-        <v>181</v>
+        <v>167</v>
       </c>
       <c r="G85" t="s">
-        <v>125</v>
+        <v>113</v>
       </c>
       <c r="H85" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="I85" t="s">
-        <v>182</v>
+        <v>168</v>
       </c>
       <c r="J85">
         <v>36</v>
@@ -3085,7 +3074,7 @@
     </row>
     <row r="86" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
-        <v>121</v>
+        <v>110</v>
       </c>
       <c r="C86">
         <v>53.739739</v>
@@ -3094,19 +3083,19 @@
         <v>-2.1832582999999999</v>
       </c>
       <c r="E86" s="1" t="s">
-        <v>113</v>
+        <v>104</v>
       </c>
       <c r="F86" t="s">
-        <v>112</v>
+        <v>103</v>
       </c>
       <c r="G86" t="s">
-        <v>82</v>
+        <v>74</v>
       </c>
       <c r="H86" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="I86" t="s">
-        <v>133</v>
+        <v>120</v>
       </c>
       <c r="J86">
         <v>36</v>
@@ -3114,7 +3103,7 @@
     </row>
     <row r="87" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
-        <v>121</v>
+        <v>110</v>
       </c>
       <c r="C87">
         <v>53.745179999999998</v>
@@ -3123,19 +3112,19 @@
         <v>-2.1223703999999999</v>
       </c>
       <c r="E87" s="1" t="s">
-        <v>114</v>
+        <v>105</v>
       </c>
       <c r="F87" t="s">
-        <v>112</v>
+        <v>103</v>
       </c>
       <c r="G87" t="s">
-        <v>82</v>
+        <v>74</v>
       </c>
       <c r="H87" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="I87" t="s">
-        <v>183</v>
+        <v>169</v>
       </c>
       <c r="J87">
         <v>36</v>
@@ -3143,7 +3132,7 @@
     </row>
     <row r="88" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
-        <v>115</v>
+        <v>106</v>
       </c>
       <c r="C88" s="1">
         <v>53.769137999999998</v>
@@ -3152,13 +3141,13 @@
         <v>-2.1654163999999998</v>
       </c>
       <c r="E88" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H88" t="s">
+        <v>108</v>
+      </c>
+      <c r="I88" t="s">
         <v>119</v>
-      </c>
-      <c r="I88" t="s">
-        <v>132</v>
       </c>
       <c r="J88">
         <v>36</v>
@@ -3166,7 +3155,7 @@
     </row>
     <row r="89" spans="1:10" ht="34" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
-        <v>115</v>
+        <v>106</v>
       </c>
       <c r="C89">
         <v>53.753045999999998</v>
@@ -3175,13 +3164,13 @@
         <v>-2.1947424</v>
       </c>
       <c r="E89" s="1" t="s">
-        <v>116</v>
+        <v>176</v>
       </c>
       <c r="H89" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="I89" t="s">
-        <v>184</v>
+        <v>170</v>
       </c>
       <c r="J89">
         <v>36</v>
@@ -3189,18 +3178,18 @@
     </row>
     <row r="90" spans="1:10" ht="34" x14ac:dyDescent="0.2">
       <c r="A90" t="s">
-        <v>123</v>
+        <v>112</v>
       </c>
       <c r="B90" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C90" s="1"/>
       <c r="D90" s="1"/>
       <c r="E90" s="1" t="s">
-        <v>124</v>
+        <v>177</v>
       </c>
       <c r="H90" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="J90">
         <v>36</v>
@@ -3208,7 +3197,7 @@
     </row>
     <row r="91" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="A91" t="s">
-        <v>126</v>
+        <v>114</v>
       </c>
       <c r="C91" s="1">
         <v>53.741953600000002</v>
@@ -3217,16 +3206,16 @@
         <v>-2.1871551</v>
       </c>
       <c r="E91" s="1" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="F91" t="s">
-        <v>179</v>
+        <v>165</v>
       </c>
       <c r="H91" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="I91" t="s">
-        <v>141</v>
+        <v>128</v>
       </c>
       <c r="J91">
         <v>32</v>
@@ -3234,7 +3223,7 @@
     </row>
     <row r="92" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="A92" t="s">
-        <v>126</v>
+        <v>114</v>
       </c>
       <c r="C92" s="1">
         <v>53.754627999999997</v>
@@ -3243,36 +3232,36 @@
         <v>-2.1937121999999998</v>
       </c>
       <c r="E92" s="1" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="F92" t="s">
-        <v>179</v>
+        <v>165</v>
       </c>
       <c r="H92" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="I92" t="s">
-        <v>139</v>
+        <v>126</v>
       </c>
       <c r="J92">
         <v>32</v>
       </c>
     </row>
-    <row r="93" spans="1:10" ht="34" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="A93" t="s">
-        <v>126</v>
+        <v>114</v>
       </c>
       <c r="B93" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E93" s="1" t="s">
-        <v>127</v>
+        <v>178</v>
       </c>
       <c r="F93" t="s">
-        <v>179</v>
+        <v>165</v>
       </c>
       <c r="H93" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="J93">
         <v>32</v>
@@ -3280,7 +3269,7 @@
     </row>
     <row r="94" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="A94" t="s">
-        <v>128</v>
+        <v>115</v>
       </c>
       <c r="C94" s="1">
         <v>53.741953600000002</v>
@@ -3289,16 +3278,16 @@
         <v>-2.1871551</v>
       </c>
       <c r="E94" s="1" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="F94" t="s">
-        <v>180</v>
+        <v>166</v>
       </c>
       <c r="H94" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="I94" t="s">
-        <v>141</v>
+        <v>128</v>
       </c>
       <c r="J94">
         <v>32</v>
@@ -3306,7 +3295,7 @@
     </row>
     <row r="95" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="A95" t="s">
-        <v>128</v>
+        <v>115</v>
       </c>
       <c r="C95" s="1">
         <v>53.740279999999998</v>
@@ -3315,16 +3304,16 @@
         <v>-2.18194</v>
       </c>
       <c r="E95" s="1" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="F95" t="s">
-        <v>180</v>
+        <v>166</v>
       </c>
       <c r="H95" t="s">
-        <v>119</v>
+        <v>108</v>
       </c>
       <c r="I95" t="s">
-        <v>134</v>
+        <v>121</v>
       </c>
       <c r="J95">
         <v>32</v>

</xml_diff>